<commit_message>
Update thesis forecasting outputs and scripts
</commit_message>
<xml_diff>
--- a/Thesis Forecasting/metadata/overall_comparison/best_model_summary.xlsx
+++ b/Thesis Forecasting/metadata/overall_comparison/best_model_summary.xlsx
@@ -418,7 +418,7 @@
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RBFNN</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -476,19 +476,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>158</v>
+        <v>234</v>
       </c>
       <c r="D2" t="n">
-        <v>3.475919113707131</v>
+        <v>3.377216762221778</v>
       </c>
       <c r="E2" t="n">
-        <v>1.840847984937388</v>
+        <v>1.83697522051419</v>
       </c>
       <c r="F2" t="n">
-        <v>3.440295102101322</v>
+        <v>3.3902379831123</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8988599585985897</v>
+        <v>0.9017817700204243</v>
       </c>
     </row>
     <row r="3">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>169</v>
+        <v>265</v>
       </c>
       <c r="D3" t="n">
         <v>1.372393407127368</v>
@@ -530,19 +530,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>169</v>
+        <v>265</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6106872916793786</v>
+        <v>0.6106872916782813</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6974508930056273</v>
+        <v>0.6974508930041152</v>
       </c>
       <c r="F4" t="n">
-        <v>3.077447039614186</v>
+        <v>3.07744703961429</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9453153141242143</v>
+        <v>0.9453153141242105</v>
       </c>
     </row>
     <row r="5">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>168</v>
+        <v>244</v>
       </c>
       <c r="D5" t="n">
         <v>4.039603029011061</v>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>171</v>
+        <v>307</v>
       </c>
       <c r="D6" t="n">
         <v>1.404527208907398</v>
@@ -602,7 +602,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RBFNN</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -611,19 +611,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>168</v>
+        <v>244</v>
       </c>
       <c r="D7" t="n">
-        <v>4.209301696521237</v>
+        <v>3.852817953240654</v>
       </c>
       <c r="E7" t="n">
-        <v>1.490988678325157</v>
+        <v>1.354018360421051</v>
       </c>
       <c r="F7" t="n">
-        <v>2.254351155379669</v>
+        <v>1.948228090654059</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9046698091595458</v>
+        <v>0.9288021413168979</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update day-ahead forecasting outputs and plots
</commit_message>
<xml_diff>
--- a/Thesis Forecasting/metadata/overall_comparison/best_model_summary.xlsx
+++ b/Thesis Forecasting/metadata/overall_comparison/best_model_summary.xlsx
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RBFNN</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -509,16 +509,16 @@
         <v>203</v>
       </c>
       <c r="D2" t="n">
-        <v>5.793521167859188</v>
+        <v>5.815498951255169</v>
       </c>
       <c r="E2" t="n">
-        <v>3.18322446163071</v>
+        <v>3.178357148433609</v>
       </c>
       <c r="F2" t="n">
-        <v>7.967810392425083</v>
+        <v>8.03495817340387</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4855949283007271</v>
+        <v>0.4768882188913155</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RBFNN</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -553,16 +553,16 @@
         <v>234</v>
       </c>
       <c r="D3" t="n">
-        <v>5.503947012698498</v>
+        <v>5.365430256508413</v>
       </c>
       <c r="E3" t="n">
-        <v>4.618375436582778</v>
+        <v>4.435603963414637</v>
       </c>
       <c r="F3" t="n">
-        <v>11.22967598524945</v>
+        <v>11.56245184173678</v>
       </c>
       <c r="G3" t="n">
-        <v>0.516724948633329</v>
+        <v>0.4876581898627955</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -597,16 +597,16 @@
         <v>234</v>
       </c>
       <c r="D4" t="n">
-        <v>2.257292839824642</v>
+        <v>2.257958702419534</v>
       </c>
       <c r="E4" t="n">
-        <v>2.411839192371335</v>
+        <v>2.412928237062234</v>
       </c>
       <c r="F4" t="n">
-        <v>7.954289216601523</v>
+        <v>7.953867317844638</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6351548356956079</v>
+        <v>0.6351935377429914</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RBFNN</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -641,16 +641,16 @@
         <v>213</v>
       </c>
       <c r="D5" t="n">
-        <v>6.914546868482034</v>
+        <v>6.892833286714121</v>
       </c>
       <c r="E5" t="n">
-        <v>2.628291897104535</v>
+        <v>2.605220520308225</v>
       </c>
       <c r="F5" t="n">
-        <v>3.775856572479338</v>
+        <v>3.826593723783812</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7252522406759934</v>
+        <v>0.7178189203188657</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -685,16 +685,16 @@
         <v>276</v>
       </c>
       <c r="D6" t="n">
-        <v>6.942901795769707</v>
+        <v>6.941966326255017</v>
       </c>
       <c r="E6" t="n">
-        <v>5.472142688975849</v>
+        <v>5.470575399659038</v>
       </c>
       <c r="F6" t="n">
-        <v>16.54079834570621</v>
+        <v>16.53993398154544</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9188709960649202</v>
+        <v>0.9188794748782994</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -729,16 +729,16 @@
         <v>213</v>
       </c>
       <c r="D7" t="n">
-        <v>6.65501983293405</v>
+        <v>6.778516069692492</v>
       </c>
       <c r="E7" t="n">
-        <v>2.263569947475957</v>
+        <v>2.326595256288697</v>
       </c>
       <c r="F7" t="n">
-        <v>3.267329231872592</v>
+        <v>3.291372438935524</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8032523451372638</v>
+        <v>0.8003460879679845</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update thesis metrics and figures
</commit_message>
<xml_diff>
--- a/Thesis Forecasting/metadata/overall_comparison/best_model_summary.xlsx
+++ b/Thesis Forecasting/metadata/overall_comparison/best_model_summary.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$G$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -425,11 +425,6 @@
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,31 +463,6 @@
           <t>testing_R2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>evaluation_type</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>mape_rows_included</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>mape_rows_excluded</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>mape_rows_excluded_fraction</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>low_load_regime</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -520,23 +490,6 @@
       <c r="G2" t="n">
         <v>0.4768882188913155</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>rolling_24h_day_ahead_backtest</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>1944</v>
-      </c>
-      <c r="J2" t="n">
-        <v>24</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.01219512195121951</v>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -564,23 +517,6 @@
       <c r="G3" t="n">
         <v>0.4876581898627955</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>rolling_24h_day_ahead_backtest</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>1968</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -608,23 +544,6 @@
       <c r="G4" t="n">
         <v>0.6351935377429914</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>rolling_24h_day_ahead_backtest</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>1968</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -652,23 +571,6 @@
       <c r="G5" t="n">
         <v>0.7178189203188657</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>rolling_24h_day_ahead_backtest</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>1968</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -696,23 +598,6 @@
       <c r="G6" t="n">
         <v>0.9188794748782994</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>rolling_24h_day_ahead_backtest</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>1968</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -740,26 +625,9 @@
       <c r="G7" t="n">
         <v>0.8003460879679845</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>rolling_24h_day_ahead_backtest</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>1968</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="b">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
+  <autoFilter ref="A1:G7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>